<commit_message>
fix(deliver): 3DMine-matching colors (cross 138, trail/grid per level), grid phase anchored to block bbox, report hole-grade stats, report PNG embedded in DXF
</commit_message>
<xml_diff>
--- a/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_v2/3940平台 1008炮孔数据报告.xlsx
+++ b/北部山头3940平台2026/7、单日数据/北部山头3940平台-1008/二次圈矿成果_3940_1008_v2/3940平台 1008炮孔数据报告.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,6 +637,78 @@
         <v>101.349</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>炮孔品位统计（孔数）</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>≥3</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>1.5-3</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>1-1.5</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>0.5-1</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>&lt;0.5</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>合计孔数</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>

</xml_diff>